<commit_message>
fixed frontend tab login
</commit_message>
<xml_diff>
--- a/loi gap phai khi build.xlsx
+++ b/loi gap phai khi build.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\phat5019\key\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA6DCB6-0EFC-4994-9B23-1444457AD9D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E51EDB-8136-403A-8706-D22AD2CD3723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1965" yWindow="2100" windowWidth="25575" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <r>
       <t>t</t>
@@ -421,6 +421,14 @@
   </si>
   <si>
     <t xml:space="preserve">khong login cung luc 2 tk </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>git rm --cached -- tist_device_tokens.ps1</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>loai bo file de up len git chu khong xoa file</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -770,10 +778,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="104.125" customWidth="1"/>
+    <col min="2" max="2" width="35.25" customWidth="1"/>
+    <col min="3" max="3" width="118.625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="32.25" customHeight="1">
@@ -807,7 +816,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="409.5">
+    <row r="10" spans="1:4" ht="33" customHeight="1">
       <c r="A10">
         <v>3</v>
       </c>
@@ -829,7 +838,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="409.5">
+    <row r="12" spans="1:4" ht="28.5" customHeight="1">
       <c r="A12">
         <v>5</v>
       </c>
@@ -854,6 +863,14 @@
       </c>
       <c r="B14" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>